<commit_message>
update the status of rFRObservationLaboratoryReportResultsDocument ca32606e83d713a66165bbf9112272eaeda6dbcf
</commit_message>
<xml_diff>
--- a/FixIssues/ig/StructureDefinition-fr-observation-laboratory-report-results-document.xlsx
+++ b/FixIssues/ig/StructureDefinition-fr-observation-laboratory-report-results-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T08:03:44+00:00</t>
+    <t>2026-06-22T08:16:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -598,7 +598,8 @@
   <si>
     <t>Niveau de complétude :
 - 'final' si le résultat est présent
-- 'cancelled' dans le cas où l'élément d'examen n’a pu être et ne sera pas réalisé</t>
+- 'cancelled' dans le cas où l'élément d'examen n’a pu être et ne sera pas réalisé
+- 'registered' le résultat n'est pas encore disponible et est attendu</t>
   </si>
   <si>
     <t>The status of the result value.</t>

</xml_diff>